<commit_message>
Align dashboard, AI analysis, mobile table, and analytics updates
</commit_message>
<xml_diff>
--- a/validTickersXLS/preferite.xlsx
+++ b/validTickersXLS/preferite.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B74"/>
+  <dimension ref="A1:B68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -623,682 +623,610 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>A2A.MI</t>
+          <t>AIGG.MI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>A2A</t>
+          <t>WISDOMTREE GRAINS.MI</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>AIGG.MI</t>
+          <t>ALAT.MI</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>WISDOMTREE GRAINS.MI</t>
+          <t>AMUNDI MSCI LATIN AMERICA EMER UCITS ETF.MI</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ALAT.MI</t>
+          <t>ALUM.MI</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>AMUNDI MSCI LATIN AMERICA EMER UCITS ETF.MI</t>
+          <t>ETFS ALUMINIUM</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ALUM.MI</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>ETFS ALUMINIUM</t>
-        </is>
-      </c>
+          <t>AVIO.MI</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>AVIO.MI</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr"/>
+          <t>BAMI.MI</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Banco Bpm</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>BAMI.MI</t>
+          <t>BATT.MI</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Banco Bpm</t>
+          <t>L&amp;G BATTERY VALUE-CHAIN UCITS ETF.MI</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>BATT.MI</t>
+          <t>BKCH.MI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>L&amp;G BATTERY VALUE-CHAIN UCITS ETF.MI</t>
+          <t>GLOBAL X BLOCKCHAIN UCITS ETF.MI</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>BKCH.MI</t>
+          <t>BMED.MI</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>GLOBAL X BLOCKCHAIN UCITS ETF.MI</t>
+          <t>Banca Mediolanum</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>BMED.MI</t>
+          <t>BNKE.MI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Banca Mediolanum</t>
+          <t>Amundi Euro Stoxx Banks UCITS ETF Acc.MI</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>BNKE.MI</t>
+          <t>BRA.MI</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Amundi Euro Stoxx Banks UCITS ETF Acc.MI</t>
+          <t>Amundi MSCI Brazil UCITS ETF Acc.MI</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>BRA.MI</t>
+          <t>BRES.MI</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Amundi MSCI Brazil UCITS ETF Acc.MI</t>
+          <t>LYXOR STX EU600 BASIC RESOURCE UCITS ETF.MI</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>BRES.MI</t>
+          <t>BRNT.MI</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>LYXOR STX EU600 BASIC RESOURCE UCITS ETF.MI</t>
+          <t>ETFS BRENT CRUDE</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>BRNT.MI</t>
+          <t>BTC-USD</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>ETFS BRENT CRUDE</t>
+          <t>Bitcoin</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>BTC-USD</t>
+          <t>COCO.MI</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Bitcoin</t>
+          <t>WISDOMTREE COCOA.MI</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>COCO.MI</t>
+          <t>COMO.MI</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>WISDOMTREE COCOA.MI</t>
+          <t>Amndi Bloom Eq-wgh Cmd ex-Agr UCITS ETF.MI</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>COMO.MI</t>
+          <t>CPR.MI</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Amndi Bloom Eq-wgh Cmd ex-Agr UCITS ETF.MI</t>
+          <t>Campari</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CPR.MI</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Campari</t>
+          <t>Cisco Systems, Inc.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>DAPP.MI</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Cisco Systems, Inc.</t>
+          <t>Blockchain</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>DAPP.MI</t>
+          <t>DFNS.MI</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Blockchain</t>
+          <t>VanEck Defense UCITS ETF.MI</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>DFNS.MI</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>VanEck Defense UCITS ETF.MI</t>
-        </is>
-      </c>
+          <t>DOGE-USD</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>DOGE-USD</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr"/>
+          <t>ENEL.MI</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Enel</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ENEL.MI</t>
+          <t>ENI.MI</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Enel</t>
+          <t>Eni</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ENI.MI</t>
+          <t>ESPO.MI</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Eni</t>
+          <t>Video Gaming</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ESPO.MI</t>
+          <t>ETH-USD</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Video Gaming</t>
+          <t>Etherium</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ETH-USD</t>
+          <t>FCRU.MI</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Etherium</t>
+          <t>WISDOMTREE WTI CRUDE OIL LONGER DATED.MI</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>FCRU.MI</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>WISDOMTREE WTI CRUDE OIL LONGER DATED.MI</t>
-        </is>
-      </c>
+          <t>FCT.MI</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>FCT.MI</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr"/>
+          <t>GDXJ.MI</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>oro</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>GDXJ.MI</t>
+          <t>HTWO.MI</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>oro</t>
+          <t>L&amp;G HYDROGEN ECONOMY UCITS ETF.MI</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>HTWO.MI</t>
+          <t>IAPD.MI</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>L&amp;G HYDROGEN ECONOMY UCITS ETF.MI</t>
+          <t>ISHARES ASIA PACIF DIVID UCITS ETF DIST.MI</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>IAPD.MI</t>
+          <t>IBIT</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ISHARES ASIA PACIF DIVID UCITS ETF DIST.MI</t>
+          <t>Blackrock bitcoin</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>IBIT</t>
+          <t>IBZL.MI</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Blackrock bitcoin</t>
+          <t>ISHARES MSCI BRAZIL UCITS ETF DIST.MI</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>IBZL.MI</t>
+          <t>IG.MI</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>ISHARES MSCI BRAZIL UCITS ETF DIST.MI</t>
+          <t>Italgas</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>IG.MI</t>
+          <t>INDI.MI</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Italgas</t>
+          <t>Amundi MSCI India II UCITS ETF.MI</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>INDI.MI</t>
+          <t>INRG.MI</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Amundi MSCI India II UCITS ETF.MI</t>
+          <t>ISHARES GLOBAL CLEAN ENERGY UCITS ETF.MI</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>INRG.MI</t>
+          <t>LAFRI.MI</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>ISHARES GLOBAL CLEAN ENERGY UCITS ETF.MI</t>
+          <t>Amundi Pan Africa UCITS ETF Acc.MI</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>IP.MI</t>
+          <t>LCOC.MI</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Interpump Group</t>
+          <t>WISDOMTREE COCOA 2X DAILY LEVERAGED.MI</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ISF.MI</t>
+          <t>LCOP.MI</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>FTSE100</t>
+          <t>ETFS LEVERAGED COPPER</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>JEGA.MI</t>
+          <t>LITU.MI</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>JPM Glob Equity Prem Income UCITS ETF.MI</t>
+          <t>GLOBAL X LITHIUM &amp; BATTERY TEC UCITS ETF.MI</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>JZXN</t>
+          <t>LNGA.MI</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Giusy holding car vitcoin</t>
+          <t>WISDOMTREE NATURAL GAS 2X DAILY LEV.MI</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>LAFRI.MI</t>
+          <t>LOCK.MI</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Amundi Pan Africa UCITS ETF Acc.MI</t>
+          <t>ISHARES DIGITAL SECURITY UCITS ETF ACC.MI</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>LCOC.MI</t>
+          <t>LOIL.MI</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>WISDOMTREE COCOA 2X DAILY LEVERAGED.MI</t>
+          <t>Loil</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>LCOP.MI</t>
+          <t>LPLA.MI</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>ETFS LEVERAGED COPPER</t>
+          <t>WISDOMTREE PLATINUM 2X DAILY LEVERAGED.MI</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>LDO.MI</t>
+          <t>PHPM.MI</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Leonardo</t>
+          <t>WISDOMTREE PHYSICAL PRECIOUS METALS.MI</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>LITU.MI</t>
+          <t>PHPT.MI</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>GLOBAL X LITHIUM &amp; BATTERY TEC UCITS ETF.MI</t>
+          <t>WISDOMTREE PHYSICAL PLATINUM.MI</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>LNGA.MI</t>
+          <t>REMX.MI</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>WISDOMTREE NATURAL GAS 2X DAILY LEV.MI</t>
+          <t>VANECK RARE EARTH AND METALS UCITS ETF.MI</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>LOCK.MI</t>
+          <t>SOL-USD</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>ISHARES DIGITAL SECURITY UCITS ETF ACC.MI</t>
+          <t>Solana</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>LOIL.MI</t>
+          <t>SOLR.MI</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Loil</t>
+          <t>INVESCO SOLAR ENERGY UCITS ETF ACC.MI</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>LPLA.MI</t>
+          <t>SSIL.MI</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>WISDOMTREE PLATINUM 2X DAILY LEVERAGED.MI</t>
+          <t>WISDOMTREE SILVER 1X DAILY SHORT.MI</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>PHPM.MI</t>
+          <t>U3O8.MI</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>WISDOMTREE PHYSICAL PRECIOUS METALS.MI</t>
+          <t>SPROTT URANIUM MINERS UCITS ETF.MI</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>PHPT.MI</t>
+          <t>VOD.L</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>WISDOMTREE PHYSICAL PLATINUM.MI</t>
+          <t>Vodafone</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>REMX.MI</t>
+          <t>WCLD.MI</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>VANECK RARE EARTH AND METALS UCITS ETF.MI</t>
+          <t>WISDOMTREE CLOUD COMPUT UCITS ETF USD A.MI</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>SOL-USD</t>
+          <t>WQTM.MI</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
-        <is>
-          <t>Solana</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>SOLR.MI</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>INVESCO SOLAR ENERGY UCITS ETF ACC.MI</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>SSIL.MI</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>WISDOMTREE SILVER 1X DAILY SHORT.MI</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>U3O8.MI</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>SPROTT URANIUM MINERS UCITS ETF.MI</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>VOD.L</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>Vodafone</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>WCLD.MI</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>WISDOMTREE CLOUD COMPUT UCITS ETF USD A.MI</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>WQTM.MI</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
         <is>
           <t>Windows tre quantum computing</t>
         </is>

</xml_diff>